<commit_message>
Update New Relic report - 2026-10-11 13:50:59
</commit_message>
<xml_diff>
--- a/output/proactive_report.xlsx
+++ b/output/proactive_report.xlsx
@@ -557,7 +557,9 @@
           <t>latest value</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n"/>
+      <c r="D3" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="7" t="n"/>
@@ -703,7 +705,9 @@
           <t>trend</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n"/>
+      <c r="D12" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="8" t="n"/>
@@ -717,7 +721,9 @@
           <t>trend</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n"/>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -736,7 +742,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -895,7 +901,9 @@
           <t>latest value</t>
         </is>
       </c>
-      <c r="D24" s="6" t="n"/>
+      <c r="D24" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="7" t="n"/>
@@ -974,7 +982,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">

</xml_diff>